<commit_message>
File was not complete for pdf add that and adjust names
Signed-off-by: SirGankalot <73303677+SirGankalot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Deliverables/sprint-09/planning-documents.xlsx
+++ b/Deliverables/sprint-09/planning-documents.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="448">
   <si>
     <t>Project Name</t>
   </si>
@@ -747,10 +747,37 @@
     <t>Model Optimization and Improvement for Timeseries Forecasting</t>
   </si>
   <si>
-    <t>Perform Data Preprocessing of additional Opensource Dataset</t>
-  </si>
-  <si>
-    <t>Integrate Visualization into the Pipeline</t>
+    <t>Optimization and Improvement of Anomaly Detection Approach</t>
+  </si>
+  <si>
+    <t>Timeseries Forecasting Improvement with Other Models (Person 1)</t>
+  </si>
+  <si>
+    <t>Integrate Timeseries Forecasting Results Visualization into the SDK</t>
+  </si>
+  <si>
+    <t>Apply Timeseries Decomposition on shell Dataset</t>
+  </si>
+  <si>
+    <t>Timeseries Forecasting Improvement with Other Models (Person 2)</t>
+  </si>
+  <si>
+    <t>Based on Customer Feedback add changes to preprocessing</t>
+  </si>
+  <si>
+    <t>Based on Customer Feedback add changes to feature engineering</t>
+  </si>
+  <si>
+    <t>Based on Customer Feedback add changes to Visualization</t>
+  </si>
+  <si>
+    <t>Based on Customer Feedback add suggested models</t>
+  </si>
+  <si>
+    <t>Based on Customer Feedback change library versions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing our own and new model approaches </t>
   </si>
   <si>
     <t>Timeseries Forecasting Improvement by Combining FEs from Best Models</t>
@@ -760,24 +787,6 @@
   </si>
   <si>
     <t>Timeseries Forecasting Improvement with Other Models</t>
-  </si>
-  <si>
-    <t>Based on Customer Feedback add changes to preprocessing</t>
-  </si>
-  <si>
-    <t>Based on Customer Feedback add changes to feature engineering</t>
-  </si>
-  <si>
-    <t>Based on Customer Feedback add changes to Visualization</t>
-  </si>
-  <si>
-    <t>Based on Customer Feedback add suggested models</t>
-  </si>
-  <si>
-    <t>Based on Customer Feedback change library versions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing our own and new model approaches </t>
   </si>
   <si>
     <t>Timeseries Forecasting Improvement by Trying Different Versions of Models</t>
@@ -2318,11 +2327,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1973682270"/>
-        <c:axId val="40504246"/>
+        <c:axId val="341596863"/>
+        <c:axId val="498139450"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1973682270"/>
+        <c:axId val="341596863"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2374,10 +2383,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40504246"/>
+        <c:crossAx val="498139450"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40504246"/>
+        <c:axId val="498139450"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2452,7 +2461,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1973682270"/>
+        <c:crossAx val="341596863"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2541,11 +2550,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1259645095"/>
-        <c:axId val="590118220"/>
+        <c:axId val="1492270629"/>
+        <c:axId val="144408904"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1259645095"/>
+        <c:axId val="1492270629"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2597,10 +2606,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="590118220"/>
+        <c:crossAx val="144408904"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="590118220"/>
+        <c:axId val="144408904"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2675,7 +2684,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1259645095"/>
+        <c:crossAx val="1492270629"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2764,11 +2773,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="841076318"/>
-        <c:axId val="1016926666"/>
+        <c:axId val="1136641324"/>
+        <c:axId val="1493572716"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="841076318"/>
+        <c:axId val="1136641324"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2820,10 +2829,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1016926666"/>
+        <c:crossAx val="1493572716"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1016926666"/>
+        <c:axId val="1493572716"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2898,7 +2907,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="841076318"/>
+        <c:crossAx val="1136641324"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -5053,11 +5062,11 @@
       <c r="C5" s="79"/>
       <c r="D5" s="80">
         <f>SUM(D9:D16)</f>
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E5" s="80">
         <f>D5</f>
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F5" s="79"/>
       <c r="G5" s="79"/>
@@ -5108,7 +5117,7 @@
       </c>
       <c r="E9" s="80">
         <f>$D$5</f>
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F9" s="80">
         <f>SUM(F21:F27)</f>
@@ -5116,7 +5125,7 @@
       </c>
       <c r="G9" s="80">
         <f>$D$5-F9</f>
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
@@ -5133,7 +5142,7 @@
       </c>
       <c r="E10" s="86">
         <f t="shared" ref="E10:E16" si="2">E9-D9</f>
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F10" s="86">
         <f>SUM(F28:F34)</f>
@@ -5141,7 +5150,7 @@
       </c>
       <c r="G10" s="86">
         <f t="shared" ref="G10:G16" si="3">G9-F10</f>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11">
@@ -5155,11 +5164,11 @@
       <c r="C11" s="106"/>
       <c r="D11" s="80">
         <f>SUM(D35:D41)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E11" s="80">
         <f t="shared" si="2"/>
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F11" s="80">
         <f>SUM(F35:F41)</f>
@@ -5167,7 +5176,7 @@
       </c>
       <c r="G11" s="80">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12">
@@ -5193,7 +5202,7 @@
       </c>
       <c r="G12" s="86">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13">
@@ -5219,7 +5228,7 @@
       </c>
       <c r="G13" s="80">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14">
@@ -5245,7 +5254,7 @@
       </c>
       <c r="G14" s="86">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15">
@@ -5271,7 +5280,7 @@
       </c>
       <c r="G15" s="80">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16">
@@ -5297,7 +5306,7 @@
       </c>
       <c r="G16" s="86">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17">
@@ -5560,7 +5569,7 @@
         <v>238</v>
       </c>
       <c r="D36" s="99">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E36" s="98"/>
       <c r="F36" s="98"/>
@@ -5573,7 +5582,7 @@
         <v>239</v>
       </c>
       <c r="D37" s="100">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E37" s="79"/>
       <c r="F37" s="101"/>
@@ -5612,7 +5621,7 @@
         <v>242</v>
       </c>
       <c r="D40" s="99">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E40" s="98"/>
       <c r="F40" s="88"/>
@@ -5753,7 +5762,7 @@
       <c r="A52" s="87"/>
       <c r="B52" s="95"/>
       <c r="C52" s="88" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="D52" s="99">
         <v>3.0</v>
@@ -5766,7 +5775,7 @@
       <c r="A53" s="85"/>
       <c r="B53" s="90"/>
       <c r="C53" s="96" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="D53" s="100">
         <v>3.0</v>
@@ -5779,7 +5788,7 @@
       <c r="A54" s="97"/>
       <c r="B54" s="98"/>
       <c r="C54" s="96" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="D54" s="99">
         <v>3.0</v>
@@ -5792,7 +5801,7 @@
       <c r="A55" s="85"/>
       <c r="B55" s="90"/>
       <c r="C55" s="96" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D55" s="100">
         <v>3.0</v>
@@ -5815,7 +5824,7 @@
         <v>12.0</v>
       </c>
       <c r="B57" s="112" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C57" s="96"/>
       <c r="D57" s="100"/>
@@ -5827,7 +5836,7 @@
       <c r="A58" s="97"/>
       <c r="B58" s="98"/>
       <c r="C58" s="88" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D58" s="99">
         <v>3.0</v>
@@ -5840,7 +5849,7 @@
       <c r="A59" s="85"/>
       <c r="B59" s="90"/>
       <c r="C59" s="96" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D59" s="100">
         <v>2.0</v>
@@ -5853,7 +5862,7 @@
       <c r="A60" s="97"/>
       <c r="B60" s="98"/>
       <c r="C60" s="88" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D60" s="99">
         <v>3.0</v>
@@ -5866,7 +5875,7 @@
       <c r="A61" s="103"/>
       <c r="B61" s="112"/>
       <c r="C61" s="96" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D61" s="100">
         <v>3.0</v>
@@ -5909,7 +5918,7 @@
     <row r="65">
       <c r="A65" s="85"/>
       <c r="C65" s="107" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D65" s="100">
         <v>3.0</v>
@@ -5921,7 +5930,7 @@
     <row r="66">
       <c r="A66" s="97"/>
       <c r="C66" s="88" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D66" s="99">
         <v>3.0</v>
@@ -5933,7 +5942,7 @@
     <row r="67">
       <c r="A67" s="85"/>
       <c r="C67" s="107" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D67" s="100">
         <v>3.0</v>
@@ -5945,7 +5954,7 @@
     <row r="68">
       <c r="A68" s="97"/>
       <c r="C68" s="88" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D68" s="99">
         <v>3.0</v>
@@ -5989,7 +5998,7 @@
       <c r="A72" s="97"/>
       <c r="B72" s="98"/>
       <c r="C72" s="88" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D72" s="99">
         <v>3.0</v>
@@ -6002,7 +6011,7 @@
       <c r="A73" s="85"/>
       <c r="B73" s="90"/>
       <c r="C73" s="96" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D73" s="100">
         <v>5.0</v>
@@ -6015,7 +6024,7 @@
       <c r="A74" s="97"/>
       <c r="B74" s="98"/>
       <c r="C74" s="88" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D74" s="99">
         <v>3.0</v>
@@ -6028,7 +6037,7 @@
       <c r="A75" s="85"/>
       <c r="B75" s="90"/>
       <c r="C75" s="96" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D75" s="100">
         <v>3.0</v>
@@ -6606,19 +6615,19 @@
         <v>65</v>
       </c>
       <c r="B1" s="68" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C1" s="68" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D1" s="114" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="64"/>
       <c r="B2" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C2" s="64"/>
       <c r="D2" s="64"/>
@@ -6626,7 +6635,7 @@
     <row r="3">
       <c r="A3" s="64"/>
       <c r="B3" s="51" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C3" s="64"/>
       <c r="D3" s="64"/>
@@ -6634,7 +6643,7 @@
     <row r="4">
       <c r="A4" s="64"/>
       <c r="B4" s="44" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C4" s="64"/>
       <c r="D4" s="64"/>
@@ -6642,7 +6651,7 @@
     <row r="5">
       <c r="A5" s="64"/>
       <c r="B5" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C5" s="64"/>
       <c r="D5" s="64"/>
@@ -6650,7 +6659,7 @@
     <row r="6">
       <c r="A6" s="64"/>
       <c r="B6" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C6" s="64"/>
       <c r="D6" s="64"/>
@@ -6658,7 +6667,7 @@
     <row r="7">
       <c r="A7" s="64"/>
       <c r="B7" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C7" s="64"/>
       <c r="D7" s="64"/>
@@ -6666,7 +6675,7 @@
     <row r="8">
       <c r="A8" s="64"/>
       <c r="B8" s="9" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C8" s="64"/>
       <c r="D8" s="64"/>
@@ -6674,32 +6683,32 @@
     <row r="9">
       <c r="A9" s="64"/>
       <c r="B9" s="63" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="64"/>
       <c r="B10" s="63" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="64"/>
       <c r="B11" s="63" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D11" s="64"/>
     </row>
     <row r="12">
       <c r="A12" s="64"/>
       <c r="B12" s="63" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="64"/>
       <c r="B13" s="63" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C13" s="115"/>
       <c r="D13" s="64"/>
@@ -6707,14 +6716,14 @@
     <row r="14">
       <c r="A14" s="64"/>
       <c r="B14" s="44" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="64"/>
       <c r="B15" s="64"/>
       <c r="C15" s="115" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D15" s="64"/>
     </row>
@@ -6722,7 +6731,7 @@
       <c r="A16" s="64"/>
       <c r="B16" s="64"/>
       <c r="C16" s="51" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D16" s="64"/>
     </row>
@@ -6731,7 +6740,7 @@
       <c r="B17" s="64"/>
       <c r="C17" s="64"/>
       <c r="D17" s="44" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="18">
@@ -6739,7 +6748,7 @@
       <c r="B18" s="64"/>
       <c r="C18" s="64"/>
       <c r="D18" s="44" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19">
@@ -6747,7 +6756,7 @@
       <c r="B19" s="64"/>
       <c r="C19" s="64"/>
       <c r="D19" s="44" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20">
@@ -6755,7 +6764,7 @@
       <c r="B20" s="64"/>
       <c r="C20" s="64"/>
       <c r="D20" s="44" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21">
@@ -6763,7 +6772,7 @@
       <c r="B21" s="64"/>
       <c r="C21" s="64"/>
       <c r="D21" s="44" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22">
@@ -6771,7 +6780,7 @@
       <c r="B22" s="64"/>
       <c r="C22" s="64"/>
       <c r="D22" s="44" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -6795,34 +6804,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="61" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B1" s="61" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="63" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B2" s="116" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="63" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B3" s="116" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="63" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B4" s="116" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5">
@@ -6926,21 +6935,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="117" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B1" s="118" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C1" s="119"/>
       <c r="D1" s="120" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E1" s="119"/>
       <c r="F1" s="119"/>
       <c r="G1" s="119"/>
       <c r="H1" s="119"/>
       <c r="I1" s="120" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J1" s="119"/>
       <c r="K1" s="121"/>
@@ -6949,7 +6958,7 @@
       <c r="N1" s="119"/>
       <c r="O1" s="119"/>
       <c r="P1" s="120" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="Q1" s="119"/>
       <c r="R1" s="119"/>
@@ -6959,10 +6968,10 @@
     </row>
     <row r="2">
       <c r="A2" s="117" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B2" s="122" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="C2" s="123"/>
       <c r="D2" s="123"/>
@@ -6986,10 +6995,10 @@
     </row>
     <row r="3">
       <c r="A3" s="117" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B3" s="122" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C3" s="123"/>
       <c r="D3" s="123"/>
@@ -7013,165 +7022,165 @@
     </row>
     <row r="4">
       <c r="A4" s="117" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B4" s="122" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C4" s="123"/>
       <c r="D4" s="117" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E4" s="117" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F4" s="117" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G4" s="117" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="H4" s="123"/>
       <c r="I4" s="125" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="J4" s="125" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="K4" s="125" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="L4" s="125" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="M4" s="125" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="N4" s="125" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="O4" s="123"/>
       <c r="P4" s="125" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Q4" s="125" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="R4" s="125" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="S4" s="125" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="T4" s="126"/>
       <c r="U4" s="126"/>
     </row>
     <row r="5">
       <c r="A5" s="117" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B5" s="127" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C5" s="123"/>
       <c r="D5" s="117" t="s">
         <v>124</v>
       </c>
       <c r="E5" s="128" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F5" s="128" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="G5" s="128" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="H5" s="123"/>
       <c r="I5" s="129" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="J5" s="130" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K5" s="131" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="L5" s="130" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="M5" s="130" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="N5" s="130" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="O5" s="123"/>
       <c r="P5" s="129" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="Q5" s="130" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="R5" s="130" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="S5" s="130" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="T5" s="132"/>
       <c r="U5" s="132"/>
     </row>
     <row r="6">
       <c r="A6" s="117" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B6" s="127" t="s">
         <v>83</v>
       </c>
       <c r="C6" s="123"/>
       <c r="D6" s="117" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E6" s="128" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F6" s="128" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="H6" s="123"/>
       <c r="I6" s="129" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="J6" s="130" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K6" s="131" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="L6" s="130" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="M6" s="130" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="N6" s="130" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="O6" s="123"/>
       <c r="P6" s="129" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="Q6" s="131" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="R6" s="130" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="S6" s="130" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="T6" s="132"/>
       <c r="U6" s="132"/>
@@ -7181,48 +7190,48 @@
       <c r="B7" s="123"/>
       <c r="C7" s="123"/>
       <c r="D7" s="117" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E7" s="128" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F7" s="128" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="G7" s="128" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="H7" s="123"/>
       <c r="I7" s="129" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J7" s="130" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K7" s="130" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="L7" s="130" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M7" s="130" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="N7" s="130" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="O7" s="123"/>
       <c r="P7" s="129" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="Q7" s="131" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="R7" s="130" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="S7" s="130" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="T7" s="132"/>
       <c r="U7" s="132"/>
@@ -7232,35 +7241,35 @@
       <c r="B8" s="123"/>
       <c r="C8" s="123"/>
       <c r="D8" s="117" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E8" s="128" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F8" s="128" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G8" s="128" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="H8" s="123"/>
       <c r="I8" s="129" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="J8" s="130" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K8" s="130" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="L8" s="130" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M8" s="130" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="N8" s="130" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="O8" s="123"/>
       <c r="P8" s="123"/>
@@ -7275,35 +7284,35 @@
       <c r="B9" s="123"/>
       <c r="C9" s="123"/>
       <c r="D9" s="133" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="E9" s="128" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F9" s="134" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G9" s="128" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="H9" s="123"/>
       <c r="I9" s="129" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="J9" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K9" s="131" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="L9" s="130" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="M9" s="130" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="N9" s="130" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="O9" s="123"/>
       <c r="P9" s="123"/>
@@ -7318,35 +7327,35 @@
       <c r="B10" s="123"/>
       <c r="C10" s="123"/>
       <c r="D10" s="135" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E10" s="134" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F10" s="136" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G10" s="136" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H10" s="123"/>
       <c r="I10" s="129" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="J10" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K10" s="130" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="L10" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M10" s="130" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="N10" s="130" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="O10" s="123"/>
       <c r="P10" s="137"/>
@@ -7362,22 +7371,22 @@
       <c r="C11" s="123"/>
       <c r="H11" s="123"/>
       <c r="I11" s="129" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="J11" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K11" s="130" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="L11" s="130" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M11" s="130" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="N11" s="130" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="O11" s="123"/>
       <c r="P11" s="58"/>
@@ -7397,22 +7406,22 @@
       <c r="G12" s="138"/>
       <c r="H12" s="123"/>
       <c r="I12" s="129" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="J12" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K12" s="130" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="L12" s="130" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="M12" s="130" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="N12" s="130" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="O12" s="123"/>
       <c r="T12" s="123"/>
@@ -7423,29 +7432,29 @@
       <c r="B13" s="123"/>
       <c r="C13" s="123"/>
       <c r="D13" s="139" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="E13" s="140"/>
       <c r="F13" s="140"/>
       <c r="G13" s="140"/>
       <c r="H13" s="123"/>
       <c r="I13" s="129" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="J13" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K13" s="130" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="L13" s="130" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="M13" s="130" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="N13" s="130" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="O13" s="123"/>
       <c r="P13" s="44"/>
@@ -7463,32 +7472,32 @@
         <v>134</v>
       </c>
       <c r="E14" s="143" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F14" s="143" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="G14" s="143" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H14" s="123"/>
       <c r="I14" s="129" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="J14" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K14" s="130" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="L14" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M14" s="130" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="N14" s="130" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="O14" s="123"/>
       <c r="P14" s="44"/>
@@ -7506,22 +7515,22 @@
       <c r="G15" s="144"/>
       <c r="H15" s="123"/>
       <c r="I15" s="129" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="J15" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K15" s="130" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="L15" s="130" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M15" s="130" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="N15" s="130" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="O15" s="123"/>
       <c r="P15" s="44"/>
@@ -7536,29 +7545,29 @@
       <c r="B16" s="123"/>
       <c r="C16" s="123"/>
       <c r="D16" s="120" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="E16" s="123"/>
       <c r="F16" s="123"/>
       <c r="G16" s="123"/>
       <c r="H16" s="123"/>
       <c r="I16" s="129" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="J16" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K16" s="130" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="L16" s="130" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M16" s="130" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="N16" s="130" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="O16" s="123"/>
       <c r="P16" s="44"/>
@@ -7578,22 +7587,22 @@
       <c r="G17" s="123"/>
       <c r="H17" s="123"/>
       <c r="I17" s="129" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="J17" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K17" s="130" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="L17" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M17" s="131" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="N17" s="130" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="O17" s="123"/>
       <c r="P17" s="44"/>
@@ -7608,35 +7617,35 @@
       <c r="B18" s="123"/>
       <c r="C18" s="123"/>
       <c r="D18" s="117" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E18" s="117" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F18" s="117" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G18" s="117" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="H18" s="123"/>
       <c r="I18" s="129" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="J18" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K18" s="130" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="L18" s="130" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="M18" s="130" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="N18" s="130" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="O18" s="123"/>
       <c r="P18" s="123"/>
@@ -7651,29 +7660,29 @@
       <c r="B19" s="123"/>
       <c r="C19" s="123"/>
       <c r="D19" s="117" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="E19" s="145"/>
       <c r="F19" s="145"/>
       <c r="G19" s="145"/>
       <c r="H19" s="123"/>
       <c r="I19" s="129" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="J19" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K19" s="130" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="L19" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M19" s="130" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="N19" s="130" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="O19" s="123"/>
       <c r="P19" s="123"/>
@@ -7693,22 +7702,22 @@
       <c r="G20" s="145"/>
       <c r="H20" s="123"/>
       <c r="I20" s="129" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="J20" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K20" s="130" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="L20" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M20" s="130" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="N20" s="130" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="O20" s="123"/>
       <c r="P20" s="123"/>
@@ -7727,22 +7736,22 @@
       <c r="G21" s="145"/>
       <c r="H21" s="123"/>
       <c r="I21" s="129" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="J21" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K21" s="130" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="L21" s="130" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="M21" s="130" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="N21" s="130" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="O21" s="123"/>
       <c r="P21" s="123"/>
@@ -7762,22 +7771,22 @@
       <c r="G22" s="145"/>
       <c r="H22" s="123"/>
       <c r="I22" s="146" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="J22" s="130" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K22" s="130" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="L22" s="130" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="M22" s="130" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="N22" s="130" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="O22" s="123"/>
       <c r="P22" s="123"/>
@@ -7797,22 +7806,22 @@
       <c r="G23" s="145"/>
       <c r="H23" s="123"/>
       <c r="I23" s="147" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="J23" s="136" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K23" s="136" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="L23" s="136" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="M23" s="136" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="N23" s="136" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="O23" s="123"/>
       <c r="P23" s="123"/>
@@ -7918,7 +7927,7 @@
         <v>First Name</v>
       </c>
       <c r="C1" s="149" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="D1" s="150"/>
       <c r="E1" s="151"/>
@@ -8007,7 +8016,7 @@
         <v>0.0</v>
       </c>
       <c r="F6" s="167" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G6" s="159"/>
       <c r="H6" s="159"/>
@@ -8027,7 +8036,7 @@
         <v>1.0</v>
       </c>
       <c r="F7" s="167" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="G7" s="162"/>
       <c r="H7" s="162"/>
@@ -8047,7 +8056,7 @@
         <v>2.0</v>
       </c>
       <c r="F8" s="167" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="G8" s="159"/>
       <c r="H8" s="159"/>
@@ -8067,7 +8076,7 @@
         <v>3.0</v>
       </c>
       <c r="F9" s="167" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="G9" s="162"/>
       <c r="H9" s="162"/>
@@ -8087,7 +8096,7 @@
         <v>5.0</v>
       </c>
       <c r="F10" s="167" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G10" s="159"/>
       <c r="H10" s="159"/>
@@ -8101,7 +8110,7 @@
         <v>8.0</v>
       </c>
       <c r="F11" s="167" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="G11" s="162"/>
       <c r="H11" s="162"/>
@@ -8115,7 +8124,7 @@
         <v>13.0</v>
       </c>
       <c r="F12" s="167" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G12" s="159"/>
       <c r="H12" s="159"/>
@@ -8132,7 +8141,7 @@
     </row>
     <row r="14">
       <c r="A14" s="168" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B14" s="169"/>
       <c r="C14" s="169"/>
@@ -8154,7 +8163,7 @@
     </row>
     <row r="16">
       <c r="A16" s="171" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B16" s="172"/>
       <c r="C16" s="172"/>
@@ -8166,7 +8175,7 @@
     </row>
     <row r="17">
       <c r="A17" s="173" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="B17" s="170"/>
       <c r="C17" s="170"/>
@@ -8178,7 +8187,7 @@
     </row>
     <row r="18">
       <c r="A18" s="171" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B18" s="172"/>
       <c r="C18" s="172"/>

</xml_diff>